<commit_message>
Rectification des N/Factures dans les fichiers Excel.
</commit_message>
<xml_diff>
--- a/Documents/Acomptes/Acomptes_2404.xlsx
+++ b/Documents/Acomptes/Acomptes_2404.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dossier Dev\Informatique\Gestcom\Documents\Acomptes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WpfProject\Gestcom\Documents\Acomptes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB10EA2C-83C2-4F7D-8111-9754FA108594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2C8B60C7-7D54-4BFE-8FF1-AAE8D21959A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24390" yWindow="2685" windowWidth="21600" windowHeight="11295" firstSheet="3" activeTab="5" xr2:uid="{0E496FD6-C4C3-46D7-AD4F-CF3D98897611}"/>
+    <workbookView xWindow="4128" yWindow="3396" windowWidth="17280" windowHeight="8964" firstSheet="4" activeTab="5" xr2:uid="{698689BB-8D33-47AB-978F-6213B303DB7D}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="49">
+  <si>
+    <t>SCAF DE LA FRUITIERE DU VAL DE LOUE</t>
+  </si>
   <si>
     <t>Mr Frédéric PONCET</t>
   </si>
@@ -112,6 +115,9 @@
     <t>CAFC SALINS LES BAINS   , la somme de</t>
   </si>
   <si>
+    <t>SCAF BRESSE JURASSIENNE</t>
+  </si>
+  <si>
     <t>Mr Benoit COTE</t>
   </si>
   <si>
@@ -127,6 +133,9 @@
     <t>CAFC POLIGNY            , la somme de</t>
   </si>
   <si>
+    <t>SCAF DE LONGEVELLE</t>
+  </si>
+  <si>
     <t>Mr Johann DEVAUX</t>
   </si>
   <si>
@@ -136,7 +145,7 @@
     <t xml:space="preserve">25380  CHARMOILLE              </t>
   </si>
   <si>
-    <t>A déduire N/Facture n° 113430 du 20/05/24</t>
+    <t>A déduire N/Facture n° 113430 du 31/05/24</t>
   </si>
   <si>
     <t>PS : Nous virons ce jour, sur votre compte N° 12506 20017 11707951010 37</t>
@@ -145,6 +154,9 @@
     <t>CAFC SANCEY LE GRAND    , la somme de</t>
   </si>
   <si>
+    <t>COOPERATIVE DES MONTS DE JOUX</t>
+  </si>
+  <si>
     <t>Atelier Gd Combe Chateleu</t>
   </si>
   <si>
@@ -158,6 +170,9 @@
   </si>
   <si>
     <t xml:space="preserve">                        , la somme de</t>
+  </si>
+  <si>
+    <t>SCAF DE LAVANS VUILLAFANS</t>
   </si>
   <si>
     <t>Mr Joany LEPINE</t>
@@ -608,160 +623,165 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62E75586-E990-40D1-B437-6FAEEC6D253C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE8D0342-C28B-43C0-8136-47FD20EE5E24}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC90C1A2-782B-402E-93D7-6ACCD901F9DF}">
-  <dimension ref="A11:J47"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9C93AA7-02A1-4E83-9D96-A73DD2022A10}">
+  <dimension ref="A10:J47"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="4.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="4.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="13" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.109375" style="1" customWidth="1"/>
     <col min="10" max="10" width="16" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="11.42578125" style="1"/>
+    <col min="11" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="11" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F10" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F11" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="6:6" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F12" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="6:6" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F13" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C28" s="4">
         <v>108</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E28" s="5">
         <v>4.0110000000000001</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6700</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
         <v>26873.7</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" ht="4.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F30" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
         <v>26873.7</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F31" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
         <v>1478.05</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="4.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
         <v>28351.75</v>
       </c>
     </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="46" spans="2:10" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B46" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="47" spans="2:10" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B47" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -774,151 +794,156 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20072305-65D7-45F4-BF6C-CC7B802D103A}">
-  <dimension ref="A11:J47"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5605FC1E-6EFB-4A39-8CBD-38DEE2703F0C}">
+  <dimension ref="A10:J47"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="4.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="4.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="13" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.109375" style="1" customWidth="1"/>
     <col min="10" max="10" width="16" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="11.42578125" style="1"/>
+    <col min="11" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="11" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F10" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F11" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="6:6" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F12" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="6:6" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F13" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C28" s="4">
         <v>400</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E28" s="5">
         <v>14.763</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6700</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
         <v>98912.1</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" ht="4.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F30" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
         <v>98912.1</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F31" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
         <v>5440.17</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="4.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
         <v>104352.27</v>
       </c>
     </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="46" spans="2:10" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B46" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="47" spans="2:10" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B47" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -931,165 +956,170 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5FA9F81-7725-4CB3-A823-4680B7016743}">
-  <dimension ref="A11:J50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A06A08ED-99EB-492C-BB64-F27C1371C1C5}">
+  <dimension ref="A10:J50"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="4.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="4.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="13" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.109375" style="1" customWidth="1"/>
     <col min="10" max="10" width="16" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="11.42578125" style="1"/>
+    <col min="11" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="11" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F10" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F11" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="6:6" x14ac:dyDescent="0.2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F12" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="6:6" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F13" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C28" s="4">
         <v>626</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E28" s="5">
         <v>24.433</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6700</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
         <v>163701.1</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" ht="4.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F30" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
         <v>163701.1</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F31" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
         <v>9003.56</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="33" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" ht="4.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
       <c r="J33" s="10">
         <f>SUM(J30:J31)</f>
         <v>172704.66</v>
       </c>
     </row>
-    <row r="34" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B34" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="J34" s="10">
         <v>-2147.7800000000002</v>
       </c>
     </row>
-    <row r="36" spans="2:10" ht="15" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
       <c r="F36" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J36" s="14">
         <f>SUM(J33:J35)</f>
         <v>170556.88</v>
       </c>
     </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="40" spans="2:10" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="41" spans="2:10" x14ac:dyDescent="0.2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B41" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="43" spans="2:10" ht="15" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43" spans="2:10" x14ac:dyDescent="0.25">
       <c r="H43" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="49" spans="2:10" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="49" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B49" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="50" spans="2:10" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B50" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="J50" s="10">
         <f>+J36</f>
@@ -1102,151 +1132,156 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B681FBB3-6331-4694-A5C3-4DD909B10153}">
-  <dimension ref="A11:J47"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80A11303-7F20-434E-823F-D611AD226138}">
+  <dimension ref="A10:J47"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="4.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="4.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="13" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.109375" style="1" customWidth="1"/>
     <col min="10" max="10" width="16" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="11.42578125" style="1"/>
+    <col min="11" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="11" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F10" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F11" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="6:6" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F12" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="13" spans="6:6" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F13" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C28" s="4">
         <v>455</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E28" s="5">
         <v>17.599</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6700</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
         <v>117913.3</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" ht="4.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F30" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
         <v>117913.3</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F31" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
         <v>6485.23</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="4.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
         <v>124398.53</v>
       </c>
     </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="46" spans="2:10" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B46" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="47" spans="2:10" x14ac:dyDescent="0.2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B47" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -1259,151 +1294,156 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0275E34E-C578-4F78-9DC6-1CF74432D410}">
-  <dimension ref="A11:J47"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C905DEB-607A-4C82-B6C9-614BE19399FB}">
+  <dimension ref="A10:J47"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="4.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="4.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="13" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.109375" style="1" customWidth="1"/>
     <col min="10" max="10" width="16" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="11.42578125" style="1"/>
+    <col min="11" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="11" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F10" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F11" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="12" spans="6:6" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F12" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13" spans="6:6" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F13" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C28" s="4">
         <v>516</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E28" s="5">
         <v>20.658000000000001</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6700</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
         <v>138408.6</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" ht="4.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F30" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
         <v>138408.6</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F31" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
         <v>7612.47</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="4.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
         <v>146021.07</v>
       </c>
     </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="46" spans="2:10" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B46" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="47" spans="2:10" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B47" s="1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>

</xml_diff>